<commit_message>
Add 24_07_n3 1 part
</commit_message>
<xml_diff>
--- a/Mixed/1_zhouyf.xlsx
+++ b/Mixed/1_zhouyf.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\Mixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730F1926-CE03-4126-A295-0CC478FF73C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C56FF3-97C7-42F9-BC3C-6878BAD04C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22740" yWindow="3990" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17520" yWindow="1005" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="74">
   <si>
     <t>Fre</t>
   </si>
@@ -292,6 +292,154 @@
   </si>
   <si>
     <t>"刚…就…"一般不接人的意志，此处是例外</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>～以上(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>既然…就…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～上(に)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不仅…而且…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>おかげで</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)托…的福(2)都怪</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>～上</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>で</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">(は) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-&gt; 在…方面</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～上で</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在…之后</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～あいだに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在…期间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~ちゃんと</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>牢牢地；好好地</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ちょっと-&gt;稍微；一会儿</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>やさしい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>容易的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～ているうちに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在…过程中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>夢中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>着迷；入迷；沉醉</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -387,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -399,6 +547,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -732,7 +883,9 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A2" s="3"/>
+      <c r="A2" s="3">
+        <v>0</v>
+      </c>
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
@@ -747,7 +900,9 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A3" s="3"/>
+      <c r="A3" s="3">
+        <v>0</v>
+      </c>
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
@@ -758,7 +913,9 @@
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A4" s="3"/>
+      <c r="A4" s="3">
+        <v>0</v>
+      </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
@@ -771,7 +928,9 @@
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A5" s="3"/>
+      <c r="A5" s="3">
+        <v>0</v>
+      </c>
       <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
@@ -786,7 +945,9 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A6" s="3"/>
+      <c r="A6" s="3">
+        <v>0</v>
+      </c>
       <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
@@ -799,7 +960,9 @@
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A7" s="3"/>
+      <c r="A7" s="3">
+        <v>0</v>
+      </c>
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -810,7 +973,9 @@
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A8" s="3"/>
+      <c r="A8" s="3">
+        <v>0</v>
+      </c>
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -823,7 +988,9 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A9" s="3"/>
+      <c r="A9" s="3">
+        <v>0</v>
+      </c>
       <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
@@ -834,7 +1001,9 @@
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A10" s="3"/>
+      <c r="A10" s="3">
+        <v>0</v>
+      </c>
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -845,7 +1014,9 @@
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A11" s="3"/>
+      <c r="A11" s="3">
+        <v>0</v>
+      </c>
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -858,7 +1029,9 @@
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A12" s="3"/>
+      <c r="A12" s="3">
+        <v>0</v>
+      </c>
       <c r="B12" s="3" t="s">
         <v>32</v>
       </c>
@@ -871,7 +1044,9 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A13" s="3"/>
+      <c r="A13" s="3">
+        <v>0</v>
+      </c>
       <c r="B13" s="3" t="s">
         <v>36</v>
       </c>
@@ -882,7 +1057,9 @@
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A14" s="3"/>
+      <c r="A14" s="3">
+        <v>0</v>
+      </c>
       <c r="B14" s="3" t="s">
         <v>38</v>
       </c>
@@ -893,7 +1070,9 @@
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A15" s="3"/>
+      <c r="A15" s="3">
+        <v>0</v>
+      </c>
       <c r="B15" s="3" t="s">
         <v>40</v>
       </c>
@@ -906,7 +1085,9 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A16" s="3"/>
+      <c r="A16" s="3">
+        <v>0</v>
+      </c>
       <c r="B16" s="3" t="s">
         <v>43</v>
       </c>
@@ -917,7 +1098,9 @@
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A17" s="3"/>
+      <c r="A17" s="3">
+        <v>0</v>
+      </c>
       <c r="B17" s="3" t="s">
         <v>45</v>
       </c>
@@ -928,7 +1111,9 @@
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A18" s="3"/>
+      <c r="A18" s="3">
+        <v>0</v>
+      </c>
       <c r="B18" s="3" t="s">
         <v>47</v>
       </c>
@@ -938,8 +1123,10 @@
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A19" s="3"/>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A19" s="3">
+        <v>0</v>
+      </c>
       <c r="B19" s="3" t="s">
         <v>48</v>
       </c>
@@ -952,7 +1139,9 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A20" s="3"/>
+      <c r="A20" s="3">
+        <v>0</v>
+      </c>
       <c r="B20" s="3" t="s">
         <v>51</v>
       </c>
@@ -964,66 +1153,110 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
+    <row r="21" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A21" s="3">
+        <v>0</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
+      <c r="B22" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>57</v>
+      </c>
       <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="E22" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+      <c r="B23" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
+      <c r="B24" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="E24" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
+      <c r="B25" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
+      <c r="B26" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
+      <c r="E26" s="3" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
+      <c r="B27" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+      <c r="B28" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
+      <c r="B29" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>

</xml_diff>

<commit_message>
update zhouyf 2 3 5
</commit_message>
<xml_diff>
--- a/Mixed/1_zhouyf.xlsx
+++ b/Mixed/1_zhouyf.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\Mixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C56FF3-97C7-42F9-BC3C-6878BAD04C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A308BF7-1B94-4898-BADF-FBF9A56C03DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17520" yWindow="1005" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17520" yWindow="330" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="1-5" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="123">
   <si>
     <t>Fre</t>
   </si>
@@ -440,6 +440,275 @@
   </si>
   <si>
     <t>着迷；入迷；沉醉</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ているところ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>正在…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">原型+ところ-&gt;即将做… </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>た</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>型+ところ-&gt;</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>間に</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>后接瞬间动作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>間 -&gt; 后接持续动作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~うちに + 意志</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>趁着…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~うちに + 不加意志：在…期间/过程中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~ようとしている</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>即将…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ようとする</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>：试图…</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜ようにしている</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>努力做到…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~つつある</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>正在变化过程中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~てはじめて</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>只有…，才…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一类形容词-&gt;名词</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>「い」变为「さ」，「い」变为「み」</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ひどい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>残酷的；严重的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>くせ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>毛病；特征</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～次第</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>N+次第-&gt;取决于…；次第に-&gt;渐渐…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～から～にかけて</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从…到…（大致范围）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～にかけて-&gt;在…方面</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~をはじめ-&gt;以…为首</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~からして</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>即使只抽取一个例子都是这样的，所以整体来看也当然如此</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>さすが</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>真不愧是</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>だけ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)尽可能…(2)仅仅</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)尽…(2)仅仅(3)只要…就…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～限り(3)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>いつでも</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>随时</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>いつまでも</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>-&gt;永远</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~限りでは</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>根据…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>かぎ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>~に限って</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>いじめる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>欺负</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)偏偏…(2)特别坚信</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>ほめる</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>-&gt;赞扬，称赞</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1167,7 +1436,9 @@
       <c r="E21" s="3"/>
     </row>
     <row r="22" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A22" s="3"/>
+      <c r="A22" s="3">
+        <v>0</v>
+      </c>
       <c r="B22" s="3" t="s">
         <v>56</v>
       </c>
@@ -1180,7 +1451,9 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A23" s="3"/>
+      <c r="A23" s="3">
+        <v>0</v>
+      </c>
       <c r="B23" s="3" t="s">
         <v>58</v>
       </c>
@@ -1191,7 +1464,9 @@
       <c r="E23" s="3"/>
     </row>
     <row r="24" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A24" s="3"/>
+      <c r="A24" s="3">
+        <v>0</v>
+      </c>
       <c r="B24" s="3" t="s">
         <v>61</v>
       </c>
@@ -1204,7 +1479,9 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A25" s="3"/>
+      <c r="A25" s="3">
+        <v>0</v>
+      </c>
       <c r="B25" s="5" t="s">
         <v>63</v>
       </c>
@@ -1215,7 +1492,9 @@
       <c r="E25" s="3"/>
     </row>
     <row r="26" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A26" s="3"/>
+      <c r="A26" s="3">
+        <v>0</v>
+      </c>
       <c r="B26" s="5" t="s">
         <v>65</v>
       </c>
@@ -1228,7 +1507,9 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A27" s="3"/>
+      <c r="A27" s="3">
+        <v>0</v>
+      </c>
       <c r="B27" s="3" t="s">
         <v>68</v>
       </c>
@@ -1239,7 +1520,9 @@
       <c r="E27" s="3"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A28" s="3"/>
+      <c r="A28" s="3">
+        <v>0</v>
+      </c>
       <c r="B28" s="3" t="s">
         <v>70</v>
       </c>
@@ -1250,7 +1533,9 @@
       <c r="E28" s="3"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A29" s="3"/>
+      <c r="A29" s="3">
+        <v>0</v>
+      </c>
       <c r="B29" s="3" t="s">
         <v>72</v>
       </c>
@@ -1260,145 +1545,285 @@
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
+    <row r="30" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A30" s="3">
+        <v>0</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+      <c r="E30" s="3" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+      <c r="A31" s="3">
+        <v>0</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
+      <c r="E31" s="3" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
+      <c r="A32" s="3">
+        <v>0</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>81</v>
+      </c>
       <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
+      <c r="E32" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A33" s="3">
+        <v>0</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>84</v>
+      </c>
       <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
+      <c r="E33" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+      <c r="A34" s="3">
+        <v>0</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>87</v>
+      </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
+      <c r="A35" s="3">
+        <v>0</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
+      <c r="A36" s="3">
+        <v>0</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
+      <c r="E36" s="3" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
+      <c r="A37" s="3">
+        <v>0</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
+      <c r="A38" s="3">
+        <v>0</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
+      <c r="A39" s="3">
+        <v>0</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="A40" s="3">
+        <v>0</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
+      <c r="E40" s="3" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
+      <c r="A41" s="3">
+        <v>0</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>101</v>
+      </c>
       <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
+      <c r="E41" s="3" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
+      <c r="A42" s="3">
+        <v>0</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
+      <c r="A43" s="3">
+        <v>0</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
+      <c r="A44" s="3">
+        <v>0</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
+      <c r="A45" s="3">
+        <v>0</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
+      <c r="E45" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A46" s="3">
+        <v>0</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
+      <c r="E46" s="4" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
+      <c r="A47" s="3">
+        <v>0</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>116</v>
+      </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
+      <c r="A48" s="3">
+        <v>0</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>121</v>
+      </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
+    <row r="49" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A49" s="3">
+        <v>0</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
+      <c r="E49" s="5" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A50" s="3"/>

</xml_diff>

<commit_message>
optimize recite logic & update recite
</commit_message>
<xml_diff>
--- a/Mixed/1_zhouyf.xlsx
+++ b/Mixed/1_zhouyf.xlsx
@@ -467,16 +467,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>めまい</t>
+          <t>名词 + ぎみ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>头晕</t>
+          <t>稍微有点…的倾向</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -484,7 +484,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -501,16 +501,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>まじめに</t>
+          <t>たてもの</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>认真；诚实；正经</t>
+          <t>建筑物；房屋</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -518,16 +518,16 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>〜ようにしている</t>
+          <t>むかえる</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>努力做到…</t>
+          <t>迎接</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -535,16 +535,16 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>～かと思うと</t>
+          <t>～きる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>刚…就…;本以为…却…</t>
+          <t>把某动作做完</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -552,33 +552,37 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>~限りでは</t>
+          <t>~につけて</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>根据…</t>
+          <t>一…就…；每当…</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>~につれて-&gt;伴随着</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>むかえる</t>
+          <t>まじめに</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>迎接</t>
+          <t>认真；诚实；正经</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -586,7 +590,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -603,37 +607,33 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>差別</t>
+          <t>〜ようにしている</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>歧视；区别对待</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>さべつ</t>
-        </is>
-      </c>
+          <t>努力做到…</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>~ばかりか</t>
+          <t>めまい</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>不仅仅…还…</t>
+          <t>头晕</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -641,58 +641,50 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>~につけて</t>
+          <t>いきなり</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>一…就…；每当…</t>
+          <t>突然地</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>~につれて-&gt;伴随着</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>~ようとしている</t>
+          <t>~はもとより</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>即将…</t>
+          <t>…自不必说</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>ようとする：试图…</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>たてもの</t>
+          <t>～かと思うと</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>建筑物；房屋</t>
+          <t>刚…就…;本以为…却…</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -700,16 +692,16 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>～きる</t>
+          <t>~ばかりか</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>把某动作做完</t>
+          <t>不仅仅…还…</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -717,50 +709,58 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>名词 + ぎみ</t>
+          <t>差別</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>稍微有点…的倾向</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>歧视；区别对待</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>さべつ</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>そこで</t>
+          <t>~ようとしている</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>于是…(紧接着做出了某个动作)</t>
+          <t>即将…</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ようとする：试图…</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>～かなにか</t>
+          <t>~限りでは</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>…之类的</t>
+          <t>根据…</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -768,54 +768,54 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>いつでも</t>
+          <t>さすが</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>随时</t>
+          <t>真不愧是</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>いつまでも-&gt;永远</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>~はもとより</t>
+          <t>〜からすると</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>…自不必说</t>
+          <t>从…来看</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>〜からするば</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>くせ</t>
+          <t>それに</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>毛病；特征</t>
+          <t>此外，再加上</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -823,54 +823,54 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>～限り(3)</t>
+          <t>そこで</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>(1)尽…(2)仅仅(3)只要…就…</t>
+          <t>于是…(紧接着做出了某个动作)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>かぎ</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>さすが</t>
+          <t>いつでも</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>真不愧是</t>
+          <t>随时</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>いつまでも-&gt;永远</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>人びと</t>
+          <t>～かなにか</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>人们</t>
+          <t>…之类的</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -878,54 +878,58 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>それに</t>
+          <t>～限り(3)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>此外，再加上</t>
+          <t>(1)尽…(2)仅仅(3)只要…就…</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>かぎ</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>~てはじめて</t>
+          <t>ているところ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>只有…，才…</t>
+          <t>正在…</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>~をはじめ-&gt;以…为首</t>
+          <t>原型+ところ-&gt;即将做…    た型+ところ-&gt;刚刚</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>~からして</t>
+          <t>~をもとに</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>即使只抽取一个例子都是这样的，所以整体来看也当然如此</t>
+          <t>以…为基础</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -937,15 +941,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>～おかげで</t>
+          <t>門出</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>(1)托…的福(2)都怪</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+          <t>开始新生活</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>かどで</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
@@ -954,12 +962,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>いきなり</t>
+          <t>~たとたん（に)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>突然地</t>
+          <t>一…就…</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -971,12 +979,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ぐらい</t>
+          <t>~に限って</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>(1)程度(2)至少(3)大约</t>
+          <t>(1)偏偏…(2)特别坚信</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -988,19 +996,15 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>門出</t>
+          <t>やさしい</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>开始新生活</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>かどで</t>
-        </is>
-      </c>
+          <t>容易的</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1009,12 +1013,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>~に限って</t>
+          <t>くせ</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>(1)偏偏…(2)特别坚信</t>
+          <t>毛病；特征</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1026,12 +1030,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>~をもとに</t>
+          <t>～おかげで</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>以…为基础</t>
+          <t>(1)托…的福(2)都怪</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -1043,12 +1047,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>～あいだに</t>
+          <t>~からして</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>在…期间</t>
+          <t>即使只抽取一个例子都是这样的，所以整体来看也当然如此</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1060,54 +1064,50 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ているところ</t>
+          <t>~てはじめて</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>正在…</t>
+          <t>只有…，才…</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>原型+ところ-&gt;即将做…    た型+ところ-&gt;刚刚</t>
+          <t>~をはじめ-&gt;以…为首</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>いじめる</t>
+          <t>人びと</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>欺负</t>
+          <t>人们</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>ほめる-&gt;赞扬，称赞</t>
-        </is>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>お/ご+连用+になる</t>
+          <t>～あいだに</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>尊他语</t>
+          <t>在…期间</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1115,40 +1115,40 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>~たとたん（に)</t>
+          <t>~にあたって</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>一…就…</t>
+          <t>当…时候</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>接续：辞书形</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>来日</t>
+          <t>ぐらい</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>访日</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>らいにち</t>
-        </is>
-      </c>
+          <t>(1)程度(2)至少(3)大约</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>～ているうちに</t>
+          <t>お/ご+连用+になる</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>在…过程中</t>
+          <t>尊他语</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1174,16 +1174,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>だけ</t>
+          <t>受け取る</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>(1)尽可能…(2)仅仅</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+          <t>领取；理解；承担</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>うけとる</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>受付-&gt;うけつけ</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1191,20 +1199,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>回る</t>
+          <t>~ちゃんと</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>旋转；绕行；巡回</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>まわる</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr"/>
+          <t>牢牢地；好好地</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ちょっと-&gt;稍微；一会儿</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1212,20 +1220,20 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>~にあたって</t>
+          <t>回る</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>当…时候</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>接续：辞书形</t>
-        </is>
-      </c>
+          <t>旋转；绕行；巡回</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>まわる</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1233,24 +1241,16 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>受け取る</t>
+          <t>だけ</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>领取；理解；承担</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>うけとる</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>受付-&gt;うけつけ</t>
-        </is>
-      </c>
+          <t>(1)尽可能…(2)仅仅</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1258,20 +1258,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>中顿的三种方式</t>
+          <t>来日</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>て、连用、连用+まして</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>“连用”最正式</t>
-        </is>
-      </c>
+          <t>访日</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>らいにち</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1279,20 +1279,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>~ちゃんと</t>
+          <t>～ているうちに</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>牢牢地；好好地</t>
+          <t>在…过程中</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>ちょっと-&gt;稍微；一会儿</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1300,16 +1296,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>夢中</t>
+          <t>中顿的三种方式</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>着迷；入迷；沉醉</t>
+          <t>て、连用、连用+まして</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>“连用”最正式</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1317,12 +1317,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ひどい</t>
+          <t>～をめぐって</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>残酷的；严重的</t>
+          <t>围绕着…</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1334,18 +1334,18 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>間に</t>
+          <t>～か～ないかのうちに</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>后接瞬间动作</t>
+          <t>刚…就…</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>間 -&gt; 后接持续动作</t>
+          <t>两处接同一个动词，第一处(原型/た型)，第二处ない形</t>
         </is>
       </c>
     </row>
@@ -1355,18 +1355,18 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>〜からすると</t>
+          <t>ごちそうする</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>从…来看</t>
+          <t>(我)请客</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>〜からするば</t>
+          <t>同「おごる」</t>
         </is>
       </c>
     </row>
@@ -1376,20 +1376,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>あふれる</t>
+          <t>相次いで</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>充满；溢出</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>溢れる</t>
-        </is>
-      </c>
+          <t>相继发生</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>あいつ</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>～をめぐって</t>
+          <t>夢中</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>围绕着…</t>
+          <t>着迷；入迷；沉醉</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1414,16 +1414,20 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ごちそうになる</t>
+          <t>あふれる</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>(我)受到款待；被请客</t>
+          <t>充满；溢出</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>溢れる</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1452,12 +1456,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>断る(2)</t>
+          <t>ごちそうになる</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>提前告知;拒绝</t>
+          <t>(我)受到款待；被请客</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1490,12 +1494,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>そして</t>
+          <t>断る(2)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>而且</t>
+          <t>提前告知;拒绝</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1507,18 +1511,18 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>～か～ないかのうちに</t>
+          <t>間に</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>刚…就…</t>
+          <t>后接瞬间动作</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
-          <t>两处接同一个动词，第一处(原型/た型)，第二处ない形</t>
+          <t>間 -&gt; 后接持续动作</t>
         </is>
       </c>
     </row>
@@ -1545,12 +1549,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>やさしい</t>
+          <t>そして</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>容易的</t>
+          <t>而且</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1562,37 +1566,37 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>相次いで</t>
+          <t>ひどい</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>相继发生</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>あいつ</t>
-        </is>
-      </c>
+          <t>残酷的；严重的</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>しっかりと</t>
+          <t>いじめる</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>让“稳稳地、扎实地”这种感觉变得更强调、更正式</t>
+          <t>欺负</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ほめる-&gt;赞扬，称赞</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1600,12 +1604,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>とおり(2)</t>
+          <t>このごろ</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>和…一样;按照…</t>
+          <t>最近；近来</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1617,20 +1621,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>～から～にかけて</t>
+          <t>连用+次第</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>从…到…（大致范围）</t>
+          <t>"刚…就…"一般不接人的意志，此处是例外</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>～にかけて-&gt;在…方面</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1638,24 +1638,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>行う</t>
+          <t>とおり(2)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>做…事;举行，实行</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>おこなう</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>行なう</t>
-        </is>
-      </c>
+          <t>和…一样;按照…</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1663,20 +1655,24 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>地方</t>
+          <t>行う</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>偏远地区</t>
+          <t>做…事;举行，实行</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ちほう</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
+          <t>おこなう</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>行なう</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1684,15 +1680,19 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>たばこ</t>
+          <t>地方</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>香烟</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
+          <t>偏远地区</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ちほう</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -1701,19 +1701,15 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>及ぼす</t>
+          <t>たばこ</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>波及;影响</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>およぼす</t>
-        </is>
-      </c>
+          <t>香烟</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
@@ -1722,20 +1718,20 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ごちそうする</t>
+          <t>及ぼす</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>(我)请客</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>同「おごる」</t>
-        </is>
-      </c>
+          <t>波及;影响</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>およぼす</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1743,16 +1739,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>このごろ</t>
+          <t>～上(に)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>最近；近来</t>
+          <t>不仅…而且…</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>～上で(は) -&gt; 在…方面</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1760,16 +1760,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>一类形容词-&gt;名词</t>
+          <t>～から～にかけて</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>「い」变为「さ」，「い」变为「み」</t>
+          <t>从…到…（大致范围）</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>～にかけて-&gt;在…方面</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1832,12 +1836,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>连用+次第</t>
+          <t>でき上がります</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>"刚…就…"一般不接人的意志，此处是例外</t>
+          <t>完成</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -1849,20 +1853,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>～上(に)</t>
+          <t>一类形容词-&gt;名词</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>不仅…而且…</t>
+          <t>「い」变为「さ」，「い」变为「み」</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>～上で(は) -&gt; 在…方面</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>でき上がります</t>
+          <t>しっかりと</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>完成</t>
+          <t>让“稳稳地、扎实地”这种感觉变得更强调、更正式</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -1949,16 +1949,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ともすると</t>
+          <t>ついに</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>容易；往往</t>
+          <t>终于；最终</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -1966,16 +1966,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>にあたる</t>
+          <t>~はさておき</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>相当于</t>
+          <t>暂且不论；姑且不论</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -1983,16 +1983,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>普通形+とは</t>
+          <t>にあたる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>竟然</t>
+          <t>相当于</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -2000,16 +2000,16 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ｖた＋ところで</t>
+          <t>ともすると</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>即便…</t>
+          <t>容易；往往</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -2017,16 +2017,16 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>平均</t>
+          <t>してきまる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>へいきん</t>
+          <t>做完某事就回来</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -2034,16 +2034,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>寿命</t>
+          <t>せず</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>じゅみょう</t>
+          <t>しない正式表达</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -2051,16 +2051,16 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>こつこつ</t>
+          <t>わがまま</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>孜孜不倦；坚持不懈</t>
+          <t>任性；自私</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -2068,16 +2068,16 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ついに</t>
+          <t>とれる</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>终于；最终</t>
+          <t>收获;取得；理解；</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -2085,50 +2085,58 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>せき</t>
+          <t>～だけある</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>咳嗽</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>真不愧是…</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>常与"さすが"搭配</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>わがまま</t>
+          <t>～だけのことわある</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>任性；自私</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>真不愧是...</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>常与"さすが"搭配</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>とれる</t>
+          <t>寿命</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>收获;取得；理解；</t>
+          <t>じゅみょう</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -2136,16 +2144,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>せず</t>
+          <t>立場</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>しない正式表达</t>
+          <t>たちば</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -2153,16 +2161,16 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>さすが</t>
+          <t>平均</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>不愧是…</t>
+          <t>へいきん</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -2170,16 +2178,16 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>おば</t>
+          <t>普通形+とは</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>姨妈；姑妈；</t>
+          <t>竟然</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -2187,58 +2195,50 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>～だけのことわある</t>
+          <t>せき</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>真不愧是...</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>常与"さすが"搭配</t>
-        </is>
-      </c>
+          <t>咳嗽</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>～だけある</t>
+          <t>ｖた＋ところで</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>真不愧是…</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>常与"さすが"搭配</t>
-        </is>
-      </c>
+          <t>即便…</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>~ないことには</t>
+          <t>こつこつ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>如果不…某事就无法实现</t>
+          <t>孜孜不倦；坚持不懈</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -2246,16 +2246,16 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>~はさておき</t>
+          <t>〜ずじまいだ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>暂且不论；姑且不论</t>
+          <t>某事不了了之</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -2263,16 +2263,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>扱う</t>
+          <t>おば</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>处理；对待</t>
+          <t>姨妈；姑妈；</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -2280,16 +2280,16 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>〜ずじまいだ</t>
+          <t>~ないことには</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>某事不了了之</t>
+          <t>如果不…某事就无法实现</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -2297,7 +2297,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2314,16 +2314,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>してきまる</t>
+          <t>～ことだし</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>做完某事就回来</t>
+          <t>原因</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -2335,29 +2335,33 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>～ことだし</t>
+          <t>見舞い</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>原因</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>慰问；探望；问候</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>みまい</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>~のこととなると</t>
+          <t>ぼろぼろ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>一提到…(后续接跟平时不同态度的句子)</t>
+          <t>破烂不堪；破破烂烂</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -2365,16 +2369,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>今まで</t>
+          <t>さんざん</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>以往的</t>
+          <t>彻底地，拼命地</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -2382,16 +2386,16 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>连用型+かれる</t>
+          <t>きょうだい</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>难以…(委婉拒绝)</t>
+          <t>兄弟姐妹</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -2399,79 +2403,67 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>～あげく</t>
+          <t>~のこととなると</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>在…之后(令人遗憾的结果)</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>接续是た型</t>
-        </is>
-      </c>
+          <t>一提到…(后续接跟平时不同态度的句子)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>～きり</t>
+          <t>さすが</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>做了…后，一直处于某种状态</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>接续是た型</t>
-        </is>
-      </c>
+          <t>不愧是…</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>見舞い</t>
+          <t>扱う</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>慰问；探望；问候</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>みまい</t>
-        </is>
-      </c>
+          <t>处理；对待</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>～を思いつく</t>
+          <t>何とも言いがたい</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>相出(idea)</t>
+          <t>不知该怎么说</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -2483,12 +2475,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>きょうだい</t>
+          <t>危うい</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>兄弟姐妹</t>
+          <t>差点…</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -2500,12 +2492,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>寝たきり</t>
+          <t>今まで</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>卧床不起</t>
+          <t>以往的</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -2517,12 +2509,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>さんざん</t>
+          <t>连用型+かれる</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>彻底地，拼命地</t>
+          <t>难以…(委婉拒绝)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -2534,15 +2526,19 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>立場</t>
+          <t>～あげく</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>たちば</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>在…之后(令人遗憾的结果)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>接续是た型</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
@@ -2551,12 +2547,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>たところ、…</t>
+          <t>～を思いつく</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>在…之后</t>
+          <t>相出(idea)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -2585,12 +2581,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>危うい</t>
+          <t>きつい</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>差点…</t>
+          <t>辛苦的；严格；困难；</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -2602,12 +2598,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ぼろぼろ</t>
+          <t>文句の付けようがない</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>破烂不堪；破破烂烂</t>
+          <t>无可挑剔；完美无缺</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -2619,12 +2615,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>何とも言いがたい</t>
+          <t>せずに</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>不知该怎么说</t>
+          <t>しないで正式表达</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -2636,12 +2632,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>文句の付けようがない</t>
+          <t>寝たきり</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>无可挑剔；完美无缺</t>
+          <t>卧床不起</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -2653,15 +2649,19 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>せずに</t>
+          <t>～きり</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>しないで正式表达</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>做了…后，一直处于某种状态</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>接续是た型</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2683,16 +2683,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ホーム</t>
+          <t>たところ、…</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>站台；月台</t>
+          <t>在…之后</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -2704,12 +2704,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ありがたい</t>
+          <t>面倒を見る</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>值得感谢的</t>
+          <t>照顾；照料</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -2721,12 +2721,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>パン</t>
+          <t>名词+からなる</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>面包</t>
+          <t>由…构成</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -2738,15 +2738,19 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>~によって(2)</t>
+          <t>て・では</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>手段；原因</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
+          <t>假设</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>(1)一类形容词-&gt;くて　(2)二类形容词/名词+で　(3)动词て型</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2755,12 +2759,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>～わりに</t>
+          <t>ありがたい</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>轻微的转折，后接出乎意料的结果</t>
+          <t>值得感谢的</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -2772,12 +2776,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>たとえ悪い結果にしろ</t>
+          <t>パン</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>"にしろ"同"でも"</t>
+          <t>面包</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -2789,19 +2793,15 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>N+不足</t>
+          <t>~によって(2)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ぶそく</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>不足-&gt;ふそく</t>
-        </is>
-      </c>
+          <t>手段；原因</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2810,19 +2810,15 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>～がする</t>
+          <t>～わりに</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>(第一人称的五官)感到…</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>〜がる-&gt;(第三人称心情)感到…</t>
-        </is>
-      </c>
+          <t>轻微的转折，后接出乎意料的结果</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2831,12 +2827,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ダイヤ</t>
+          <t>たとえ悪い結果にしろ</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>列车时刻表；钻石</t>
+          <t>"にしろ"同"でも"</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -2848,15 +2844,19 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>名词+からなる</t>
+          <t>N+不足</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>由…构成</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
+          <t>ぶそく</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>不足-&gt;ふそく</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2865,12 +2865,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>でも</t>
+          <t>5つずつ</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>列举</t>
+          <t>每份五个</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -2882,12 +2882,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>~わけではない</t>
+          <t>ダイヤ</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>部分否定，并非；也不是</t>
+          <t>列车时刻表；钻石</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2899,19 +2899,15 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>连用型+がたい</t>
+          <t>~ものか</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>难以…(心理活动，而不是能力)</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>たい-&gt;想要</t>
-        </is>
-      </c>
+          <t>绝对不…</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2920,19 +2916,15 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>て・では</t>
+          <t>あり得ない</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>假设</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>(1)一类形容词-&gt;くて　(2)二类形容词/名词+で　(3)动词て型</t>
-        </is>
-      </c>
+          <t>没可能</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2941,12 +2933,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>普通形+得る・得ない</t>
+          <t>~わけではない</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>能够/不能…</t>
+          <t>部分否定，并非；也不是</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -2958,15 +2950,19 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>~につき</t>
+          <t>连用型+がたい</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>因为…</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
+          <t>难以…(心理活动，而不是能力)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>たい-&gt;想要</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2975,12 +2971,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>面倒</t>
+          <t>ホーム</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>麻烦</t>
+          <t>站台；月台</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -2992,12 +2988,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>面倒を見る</t>
+          <t>普通形+得る・得ない</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>照顾；照料</t>
+          <t>能够/不能…</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -3009,12 +3005,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>~ものか</t>
+          <t>~につき</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>绝对不…</t>
+          <t>因为…</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -3026,12 +3022,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>5つずつ</t>
+          <t>ｖている＋ところ</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>每份五个</t>
+          <t>正在…</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -3043,15 +3039,19 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ｖている＋ところ</t>
+          <t>～がする</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>正在…</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
+          <t>(第一人称的五官)感到…</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>〜がる-&gt;(第三人称心情)感到…</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
@@ -3060,15 +3060,19 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>～わけがない</t>
+          <t>姿勢</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>完全否定</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
+          <t>态度；姿态</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>しせい</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
@@ -3077,12 +3081,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>～もの(结尾)</t>
+          <t>面倒</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>原因</t>
+          <t>麻烦</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -3094,12 +3098,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>～末に</t>
+          <t>ラブレター</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>在…之后(做了某个决断)</t>
+          <t>情书</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -3111,12 +3115,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>にもかかわらず</t>
+          <t>ず</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>尽管；虽然</t>
+          <t>ない正式表达</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -3128,12 +3132,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>原型+ところ</t>
+          <t>ひどい</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>即将…</t>
+          <t>残酷的；严重的</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -3145,12 +3149,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>及ぶ</t>
+          <t>～末に</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>波及，长达</t>
+          <t>在…之后(做了某个决断)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -3162,12 +3166,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ｖた＋ところ</t>
+          <t>にもかかわらず</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>刚做完…</t>
+          <t>尽管；虽然</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -3179,12 +3183,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ずに</t>
+          <t>原型+ところ</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ないで正式表达</t>
+          <t>即将…</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -3196,12 +3200,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ラブレター</t>
+          <t>及ぶ</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>情书</t>
+          <t>波及，长达</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -3213,12 +3217,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>きつい</t>
+          <t>ｖた＋ところ</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>辛苦的；严格；困难；</t>
+          <t>刚做完…</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -3230,12 +3234,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ひどい</t>
+          <t>ずに</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>残酷的；严重的</t>
+          <t>ないで正式表达</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -3247,12 +3251,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>连用+ようがない</t>
+          <t>文句</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>(1)无法做某事….(2)完全否定</t>
+          <t>抱怨；牢骚</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -3264,12 +3268,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>としか言いようがない</t>
+          <t>～を思いだす</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>只能说是…</t>
+          <t>想起(旧事)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -3281,12 +3285,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>文句</t>
+          <t>～もの(结尾)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>抱怨；牢骚</t>
+          <t>原因</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -3298,12 +3302,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>～を思いだす</t>
+          <t>としか言いようがない</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>想起(旧事)</t>
+          <t>只能说是…</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -3315,12 +3319,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>あり得ない</t>
+          <t>でも</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>没可能</t>
+          <t>列举</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -3332,19 +3336,15 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>上昇</t>
+          <t>连用+ようがない</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>じょうしょう</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>上升；增加</t>
-        </is>
-      </c>
+          <t>(1)无法做某事….(2)完全否定</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
@@ -3353,19 +3353,15 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>上場</t>
+          <t>～わけがない</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>じょうじょう</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>上市</t>
-        </is>
-      </c>
+          <t>完全否定</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
@@ -3374,17 +3370,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>姿勢</t>
+          <t>上昇</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>态度；姿态</t>
+          <t>じょうしょう</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>しせい</t>
+          <t>上升；增加</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -3395,15 +3391,19 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>に泊まる</t>
+          <t>上場</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>临时短住</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
+          <t>じょうじょう</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
       <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
@@ -3412,12 +3412,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ず</t>
+          <t>に泊まる</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>ない正式表达</t>
+          <t>临时短住</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -3491,16 +3491,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ぬれる</t>
+          <t>ｖた＋もでだ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>淋湿；浸湿</t>
+          <t>怀念过去常做的事</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -3508,16 +3508,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>～とみえる</t>
+          <t>うわさ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>推测…</t>
+          <t>传闻；流言</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -3525,16 +3525,16 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>うわさ</t>
+          <t>ぬれる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>传闻；流言</t>
+          <t>淋湿；浸湿</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -3542,33 +3542,37 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>どうにかして</t>
+          <t>〜にきまっている</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>想方设法、无论如何</t>
+          <t>肯定....</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>〜に決まっている</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>しかる</t>
+          <t>おしゃれ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>责备；训斥；斥责</t>
+          <t>时尚</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -3576,100 +3580,92 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>〜ことはない</t>
+          <t>やはり</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>没必要做某事</t>
+          <t>果然；毕竟</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>辞书形</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>口を出す</t>
+          <t>証拠</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>插嘴；干预</t>
+          <t>证据</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>くちをだす</t>
+          <t>しょうこ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>〜にきまっている</t>
+          <t>かゆい</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>肯定....</t>
+          <t>痒</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>〜に決まっている</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>証拠</t>
+          <t>口を出す</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>证据</t>
+          <t>插嘴；干预</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>しょうこ</t>
+          <t>くちをだす</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>かゆい</t>
+          <t>しかる</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>痒</t>
+          <t>责备；训斥；斥责</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -3681,16 +3677,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>やはり</t>
+          <t>ポリシー</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>果然；毕竟</t>
+          <t>政策；方针</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3698,16 +3698,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>おしゃれ</t>
+          <t>ささえる</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>时尚</t>
+          <t>支撑；支持</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>支える</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -3715,29 +3719,33 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ｖた＋もでだ</t>
+          <t>に越したことはない</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>怀念过去常做的事</t>
+          <t>最好是…</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>辞书形</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>えさ</t>
+          <t>N+には</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>饲料</t>
+          <t>对象</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -3745,62 +3753,58 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ささえる</t>
+          <t>～とみえる</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>支撑；支持</t>
+          <t>推测…</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>支える</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>税金</t>
+          <t>〜ことはない</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ぜいきん</t>
+          <t>没必要做某事</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>辞书形</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>に越したことはない</t>
+          <t>どうにかして</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>最好是…</t>
+          <t>想方设法、无论如何</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>辞书形</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3825,12 +3829,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>N+には</t>
+          <t>気軽に</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>对象</t>
+          <t>轻松地；随意地</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -3842,20 +3846,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ポリシー</t>
+          <t>えさ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>政策；方针</t>
+          <t>饲料</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>policy</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3863,12 +3863,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>〜べきだ</t>
+          <t>税金</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>(社会常识或道德性)应该做某事</t>
+          <t>ぜいきん</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -3880,16 +3880,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>かい</t>
+          <t>~ないわけにはいかない</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>价值</t>
+          <t>(心理上)必须要做某事</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>辞书~わけにはいかない-&gt;不能做</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3897,12 +3901,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>～はずだ</t>
+          <t>〜べきだ</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>(可能形较高)推测</t>
+          <t>(社会常识或道德性)应该做某事</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -3914,20 +3918,16 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>~ないではいられない</t>
+          <t>かい</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>情不自禁做某事</t>
+          <t>价值</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>主要是第三人称的话，要接"そうだ"</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3935,12 +3935,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>気軽に</t>
+          <t>～はずだ</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>轻松地；随意地</t>
+          <t>(可能形较高)推测</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -3952,20 +3952,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>~ないわけにはいかない</t>
+          <t>大切</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>(心理上)必须要做某事</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>辞书~わけにはいかない-&gt;不能做</t>
-        </is>
-      </c>
+          <t>重要</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>たいせつ</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3973,20 +3973,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>大切</t>
+          <t>~ないではいられない</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>重要</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>たいせつ</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>情不自禁做某事</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>主要是第三人称的话，要接"そうだ"</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3994,16 +3994,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>～にすぎない</t>
+          <t>〜に相違ない</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>只不过…</t>
+          <t>肯定....</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>同"に違いない"</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4011,20 +4015,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>～かれる</t>
+          <t>主張</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>难以…(委婉否定/拒绝)</t>
+          <t>しゅちょう</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>接续：连用型</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4032,12 +4032,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>～ぐらい</t>
+          <t>〜というものだ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>(1)最低程度…(2)大约，左右</t>
+          <t>从常识开看，简直是…</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -4049,12 +4049,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>～まい</t>
+          <t>出張</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>"ない"的书面语</t>
+          <t>しゅっちょう</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -4066,12 +4066,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>断る</t>
+          <t>とんでもない</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>事先告知</t>
+          <t>不用;哪里的话</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -4083,20 +4083,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>〜に相違ない</t>
+          <t>～まい</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>肯定....</t>
+          <t>"ない"的书面语</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>同"に違いない"</t>
-        </is>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -4104,12 +4100,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>とんでもない</t>
+          <t>断る</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>不用;哪里的话</t>
+          <t>事先告知</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -4121,12 +4117,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>出張</t>
+          <t>～ぐらい</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>しゅっちょう</t>
+          <t>(1)最低程度…(2)大约，左右</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -4138,16 +4134,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>〜というものだ</t>
+          <t>～かれる</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>从常识开看，简直是…</t>
+          <t>难以…(委婉否定/拒绝)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>接续：连用型</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4155,19 +4155,15 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>引っ張る</t>
+          <t>～にすぎない</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">拖拉拽 </t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>ひっぱる</t>
-        </is>
-      </c>
+          <t>只不过…</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
@@ -4176,16 +4172,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>主張</t>
+          <t>~てしかたがない</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>しゅちょう</t>
+          <t>非常…</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>主要是第三人称的话，要接"らしい""ようだ"</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4214,20 +4214,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>~てしかたがない</t>
+          <t>を的翻译</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>非常…</t>
+          <t>把…</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>主要是第三人称的话，要接"らしい""ようだ"</t>
-        </is>
-      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -4235,15 +4231,19 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>辞书〜ものだ</t>
+          <t>引っ張る</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>(1)真理…(2)最好做…</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t xml:space="preserve">拖拉拽 </t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ひっぱる</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -4269,18 +4269,18 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>～さえ～ば・たら・なら</t>
+          <t>~ざるを得ない</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>只要…就…</t>
+          <t>接续:ない去掉</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>”さえ”甚至</t>
+          <t>特例:する-&gt;せざる</t>
         </is>
       </c>
     </row>
@@ -4290,12 +4290,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>〜ものか</t>
+          <t>〜にほかならない</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>完全否定，口语</t>
+          <t>正是…</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -4307,20 +4307,16 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>~てしょうがない</t>
+          <t>辞书〜ものだ</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>非常</t>
+          <t>(1)真理…(2)最好做…</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>主要是第三人称的话，要接"らしい""ようだ"</t>
-        </is>
-      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -4328,20 +4324,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>~ずにはいられない</t>
+          <t>なんて</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>情不自禁做某事</t>
+          <t>竟然；这样的</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>主要是第三人称的话，要接"そうだ"</t>
-        </is>
-      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -4349,12 +4341,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>大切にする</t>
+          <t>受け入れる</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>珍惜；爱护</t>
+          <t>接受</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -4366,16 +4358,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>を的翻译</t>
+          <t>~ずにはいられない</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>把…</t>
+          <t>情不自禁做某事</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>主要是第三人称的话，要接"そうだ"</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -4383,16 +4379,20 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>なんて</t>
+          <t>~てしょうがない</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>竟然；这样的</t>
+          <t>非常</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>主要是第三人称的话，要接"らしい""ようだ"</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -4400,12 +4400,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>受け入れる</t>
+          <t>〜ものか</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>接受</t>
+          <t>完全否定，口语</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -4417,16 +4417,20 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>〜にほかならない</t>
+          <t>～さえ～ば・たら・なら</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>正是…</t>
+          <t>只要…就…</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>”さえ”甚至</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4434,20 +4438,16 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>~ざるを得ない</t>
+          <t>大切にする</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>接续:ない去掉</t>
+          <t>珍惜；爱护</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>特例:する-&gt;せざる</t>
-        </is>
-      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">

</xml_diff>